<commit_message>
update, including some new plots, more complete units table, and updated colors (requires re-running smapling proccessing scripts and updating sample master files
</commit_message>
<xml_diff>
--- a/data/sampling/ic_icpms/ic_icpms_data.xlsx
+++ b/data/sampling/ic_icpms/ic_icpms_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/ECM/alhic1901_deep_layering/github/data/sampling/ic_icpms/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/ic_icpms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2978EA0-D850-324C-A856-5FEF733FCE3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEEDBC8-E036-1E4C-9C0D-DD060838F721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1020" yWindow="760" windowWidth="29220" windowHeight="18880" xr2:uid="{CFB0DC14-1812-354F-9E14-8529713485B8}"/>
   </bookViews>
@@ -71,9 +71,6 @@
     <t>Mg2+</t>
   </si>
   <si>
-    <t>Ca+</t>
-  </si>
-  <si>
     <t>LIC</t>
   </si>
   <si>
@@ -222,6 +219,9 @@
   </si>
   <si>
     <t>ICPMS</t>
+  </si>
+  <si>
+    <t>Ca2+</t>
   </si>
 </sst>
 </file>
@@ -645,147 +645,147 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="M1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" t="s">
         <v>15</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>16</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>17</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>18</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>19</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>20</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>21</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>22</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>23</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>24</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>25</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>26</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>27</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>28</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>29</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>30</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>31</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>32</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>33</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>34</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>35</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AI1" t="s">
         <v>36</v>
       </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
         <v>37</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AK1" t="s">
         <v>38</v>
       </c>
-      <c r="AK1" t="s">
+      <c r="AL1" t="s">
         <v>39</v>
       </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>40</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>41</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>42</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>43</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>44</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>45</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>46</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>47</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>48</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>49</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>50</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>51</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>52</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>53</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>54</v>
       </c>
-      <c r="BA1" t="s">
-        <v>55</v>
-      </c>
       <c r="BB1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BC1" t="s">
         <v>57</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BD1" t="s">
         <v>58</v>
-      </c>
-      <c r="BD1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>155.065</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="3" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>155.09578569999999</v>
@@ -858,10 +858,10 @@
     </row>
     <row r="4" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>155.12657139999999</v>
@@ -896,10 +896,10 @@
     </row>
     <row r="5" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>155.15735710000001</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="6" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>155.19814289999999</v>
@@ -972,10 +972,10 @@
     </row>
     <row r="7" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7">
         <v>155.24192859999999</v>
@@ -1010,10 +1010,10 @@
     </row>
     <row r="8" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8">
         <v>155.2782143</v>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="9" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9">
         <v>155.30799999999999</v>
@@ -1086,10 +1086,10 @@
     </row>
     <row r="10" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>155.065</v>
@@ -1124,10 +1124,10 @@
     </row>
     <row r="11" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11">
         <v>155.095786</v>
@@ -1162,10 +1162,10 @@
     </row>
     <row r="12" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12">
         <v>155.12657100000001</v>
@@ -1200,10 +1200,10 @@
     </row>
     <row r="13" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13">
         <v>155.15735699999999</v>
@@ -1238,10 +1238,10 @@
     </row>
     <row r="14" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14">
         <v>155.19814299999999</v>
@@ -1276,10 +1276,10 @@
     </row>
     <row r="15" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C15">
         <v>155.241929</v>
@@ -1314,10 +1314,10 @@
     </row>
     <row r="16" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16">
         <v>155.27821399999999</v>
@@ -1352,10 +1352,10 @@
     </row>
     <row r="17" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C17">
         <v>155.083</v>
@@ -1493,10 +1493,10 @@
     </row>
     <row r="18" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C18">
         <v>155.11500000000001</v>
@@ -1634,10 +1634,10 @@
     </row>
     <row r="19" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C19">
         <v>155.14699999999999</v>
@@ -1775,10 +1775,10 @@
     </row>
     <row r="20" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C20">
         <v>155.18549999999999</v>
@@ -1916,10 +1916,10 @@
     </row>
     <row r="21" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C21">
         <v>155.2165</v>
@@ -2057,10 +2057,10 @@
     </row>
     <row r="22" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C22">
         <v>155.24799999999999</v>
@@ -2198,10 +2198,10 @@
     </row>
     <row r="23" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C23">
         <v>155.286</v>
@@ -2339,10 +2339,10 @@
     </row>
     <row r="24" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C24">
         <v>156.8152</v>
@@ -2485,10 +2485,10 @@
     </row>
     <row r="25" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C25">
         <v>156.83049389999999</v>
@@ -2631,10 +2631,10 @@
     </row>
     <row r="26" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26">
         <v>156.8429984</v>
@@ -2777,10 +2777,10 @@
     </row>
     <row r="27" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C27">
         <v>156.8564025</v>
@@ -2923,10 +2923,10 @@
     </row>
     <row r="28" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C28">
         <v>156.8690622</v>
@@ -3069,10 +3069,10 @@
     </row>
     <row r="29" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C29">
         <v>156.8829236</v>
@@ -3215,10 +3215,10 @@
     </row>
     <row r="30" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C30">
         <v>156.89620719999999</v>
@@ -3361,10 +3361,10 @@
     </row>
     <row r="31" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C31">
         <v>156.91009</v>
@@ -3507,10 +3507,10 @@
     </row>
     <row r="32" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C32">
         <v>156.92437000000001</v>
@@ -3653,10 +3653,10 @@
     </row>
     <row r="33" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B33" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C33">
         <v>156.93795900000001</v>
@@ -3799,10 +3799,10 @@
     </row>
     <row r="34" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C34">
         <v>156.95110600000001</v>
@@ -3945,10 +3945,10 @@
     </row>
     <row r="35" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C35">
         <v>156.96452500000001</v>
@@ -4091,10 +4091,10 @@
     </row>
     <row r="36" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B36" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C36">
         <v>156.97749899999999</v>
@@ -4237,10 +4237,10 @@
     </row>
     <row r="37" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C37">
         <v>156.99092099999999</v>
@@ -4383,10 +4383,10 @@
     </row>
     <row r="38" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C38">
         <v>157.00419099999999</v>
@@ -4529,10 +4529,10 @@
     </row>
     <row r="39" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C39">
         <v>157.01694800000001</v>
@@ -4675,10 +4675,10 @@
     </row>
     <row r="40" spans="1:56" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C40">
         <v>157.029854</v>

</xml_diff>

<commit_message>
bring all up to date
</commit_message>
<xml_diff>
--- a/data/sampling/ic_icpms/ic_icpms_data.xlsx
+++ b/data/sampling/ic_icpms/ic_icpms_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/ic_icpms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86B2B79-D020-D542-9C8B-056954FE83C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5355A640-BBCB-1E4B-A102-DB60153BE8E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19460" yWindow="-22640" windowWidth="29160" windowHeight="18880" xr2:uid="{CFB0DC14-1812-354F-9E14-8529713485B8}"/>
+    <workbookView xWindow="240" yWindow="-21000" windowWidth="29160" windowHeight="18980" xr2:uid="{CFB0DC14-1812-354F-9E14-8529713485B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5349,6 +5349,30 @@
         <f t="shared" si="1"/>
         <v>157.02611000000002</v>
       </c>
+      <c r="F53">
+        <v>113.2410198</v>
+      </c>
+      <c r="G53">
+        <v>45.386590079999998</v>
+      </c>
+      <c r="H53">
+        <v>379.52659840000001</v>
+      </c>
+      <c r="I53">
+        <v>99.923640879999994</v>
+      </c>
+      <c r="J53">
+        <v>3.2603787440000001</v>
+      </c>
+      <c r="K53">
+        <v>16.468898970000001</v>
+      </c>
+      <c r="L53">
+        <v>100.12715710000001</v>
+      </c>
+      <c r="N53">
+        <v>18.159056700000001</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" t="s">

</xml_diff>